<commit_message>
Add subject column to stock balance report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mp3wof2iwnsjKqWXT9wGnu
</commit_message>
<xml_diff>
--- a/ostatki/ostatki_s_razmerom.xlsx
+++ b/ostatki/ostatki_s_razmerom.xlsx
@@ -673,7 +673,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:P240"/>
+  <dimension ref="A2:Q240"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.5" defaultRowHeight="11.429" customHeight="1"/>
   <cols>
     <col width="10.5" customWidth="1" style="1" min="1" max="1"/>
@@ -692,6 +692,7 @@
     <col width="14" customWidth="1" style="1" min="14" max="14"/>
     <col width="14" customWidth="1" style="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="10" customFormat="1" customHeight="1" s="1"/>
@@ -753,6 +754,11 @@
       <c r="P6" s="21" t="inlineStr">
         <is>
           <t>Размер</t>
+        </is>
+      </c>
+      <c r="Q6" s="21" t="inlineStr">
+        <is>
+          <t>Предмет</t>
         </is>
       </c>
     </row>
@@ -785,6 +791,7 @@
       <c r="N7" s="25" t="n"/>
       <c r="O7" s="26" t="n"/>
       <c r="P7" s="27" t="n"/>
+      <c r="Q7" s="27" t="n"/>
     </row>
     <row r="8" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A8" s="24" t="n"/>
@@ -835,6 +842,7 @@
         </is>
       </c>
       <c r="P8" s="26" t="n"/>
+      <c r="Q8" s="26" t="n"/>
     </row>
     <row r="9" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A9" s="10" t="inlineStr">
@@ -865,6 +873,7 @@
         <v>1154</v>
       </c>
       <c r="P9" s="21" t="n"/>
+      <c r="Q9" s="21" t="n"/>
     </row>
     <row r="10" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A10" s="13" t="inlineStr">
@@ -907,6 +916,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q10" s="13" t="inlineStr">
+        <is>
+          <t>Боди</t>
+        </is>
+      </c>
     </row>
     <row r="11" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A11" s="13" t="inlineStr">
@@ -949,6 +963,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q11" s="13" t="inlineStr">
+        <is>
+          <t>Боди</t>
+        </is>
+      </c>
     </row>
     <row r="12" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A12" s="13" t="inlineStr">
@@ -991,6 +1010,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q12" s="13" t="inlineStr">
+        <is>
+          <t>Боди</t>
+        </is>
+      </c>
     </row>
     <row r="13" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A13" s="13" t="inlineStr">
@@ -1033,6 +1057,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q13" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="14" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="13" t="inlineStr">
@@ -1075,6 +1104,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q14" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="15" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A15" s="13" t="inlineStr">
@@ -1117,6 +1151,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="16" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A16" s="13" t="inlineStr">
@@ -1159,6 +1198,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="17" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A17" s="13" t="inlineStr">
@@ -1201,6 +1245,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="18" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A18" s="13" t="inlineStr">
@@ -1243,6 +1292,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="19" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A19" s="13" t="inlineStr">
@@ -1285,6 +1339,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="20" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A20" s="13" t="inlineStr">
@@ -1327,6 +1386,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="Q20" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="21" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A21" s="13" t="inlineStr">
@@ -1369,6 +1433,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="22" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A22" s="13" t="inlineStr">
@@ -1411,6 +1480,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="23" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A23" s="13" t="inlineStr">
@@ -1453,6 +1527,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q23" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="24" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A24" s="13" t="inlineStr">
@@ -1495,6 +1574,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="25" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A25" s="13" t="inlineStr">
@@ -1537,6 +1621,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="26" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A26" s="13" t="inlineStr">
@@ -1579,6 +1668,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q26" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="27" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A27" s="13" t="inlineStr">
@@ -1621,6 +1715,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q27" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="28" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A28" s="13" t="inlineStr">
@@ -1663,6 +1762,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="Q28" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="29" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A29" s="13" t="inlineStr">
@@ -1705,6 +1809,11 @@
           <t>44-46</t>
         </is>
       </c>
+      <c r="Q29" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="30" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A30" s="13" t="inlineStr">
@@ -1747,6 +1856,11 @@
           <t>52-54</t>
         </is>
       </c>
+      <c r="Q30" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="31" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A31" s="13" t="inlineStr">
@@ -1789,6 +1903,11 @@
           <t>56-58</t>
         </is>
       </c>
+      <c r="Q31" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="32" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A32" s="13" t="inlineStr">
@@ -1831,6 +1950,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q32" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="33" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A33" s="13" t="inlineStr">
@@ -1873,6 +1997,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q33" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="34" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A34" s="13" t="inlineStr">
@@ -1915,6 +2044,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q34" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="35" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A35" s="13" t="inlineStr">
@@ -1957,6 +2091,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q35" s="13" t="inlineStr">
+        <is>
+          <t>Велосипедки</t>
+        </is>
+      </c>
     </row>
     <row r="36" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A36" s="13" t="inlineStr">
@@ -1999,6 +2138,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q36" s="13" t="inlineStr">
+        <is>
+          <t>Велосипедки</t>
+        </is>
+      </c>
     </row>
     <row r="37" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A37" s="13" t="inlineStr">
@@ -2041,6 +2185,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q37" s="13" t="inlineStr">
+        <is>
+          <t>Велосипедки</t>
+        </is>
+      </c>
     </row>
     <row r="38" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A38" s="13" t="inlineStr">
@@ -2081,6 +2230,11 @@
       <c r="P38" s="13" t="inlineStr">
         <is>
           <t>48</t>
+        </is>
+      </c>
+      <c r="Q38" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
         </is>
       </c>
     </row>
@@ -2125,6 +2279,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q39" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="40" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A40" s="13" t="inlineStr">
@@ -2165,6 +2324,11 @@
       <c r="P40" s="13" t="inlineStr">
         <is>
           <t>52</t>
+        </is>
+      </c>
+      <c r="Q40" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
         </is>
       </c>
     </row>
@@ -2209,6 +2373,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q41" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="42" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A42" s="13" t="inlineStr">
@@ -2251,6 +2420,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="Q42" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="43" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A43" s="13" t="inlineStr">
@@ -2293,6 +2467,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="Q43" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="44" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A44" s="13" t="inlineStr">
@@ -2335,6 +2514,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="Q44" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="45" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A45" s="13" t="inlineStr">
@@ -2377,6 +2561,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="Q45" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="46" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A46" s="13" t="inlineStr">
@@ -2419,6 +2608,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="Q46" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="47" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A47" s="13" t="inlineStr">
@@ -2461,6 +2655,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q47" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="48" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A48" s="13" t="inlineStr">
@@ -2503,6 +2702,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q48" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="49" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A49" s="13" t="inlineStr">
@@ -2545,6 +2749,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q49" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="50" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A50" s="13" t="inlineStr">
@@ -2587,6 +2796,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q50" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="51" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A51" s="13" t="inlineStr">
@@ -2629,6 +2843,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="Q51" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="52" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A52" s="13" t="inlineStr">
@@ -2671,6 +2890,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="Q52" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="53" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A53" s="13" t="inlineStr">
@@ -2713,6 +2937,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="Q53" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="54" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A54" s="13" t="inlineStr">
@@ -2755,6 +2984,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="Q54" s="13" t="inlineStr">
+        <is>
+          <t>Туника</t>
+        </is>
+      </c>
     </row>
     <row r="55" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A55" s="13" t="inlineStr">
@@ -2797,6 +3031,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q55" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="56" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A56" s="13" t="inlineStr">
@@ -2839,6 +3078,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q56" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="57" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A57" s="13" t="inlineStr">
@@ -2881,6 +3125,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q57" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="58" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A58" s="13" t="inlineStr">
@@ -2923,6 +3172,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q58" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="59" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A59" s="13" t="inlineStr">
@@ -2965,6 +3219,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q59" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="60" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A60" s="13" t="inlineStr">
@@ -3007,6 +3266,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q60" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="61" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A61" s="13" t="inlineStr">
@@ -3049,6 +3313,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q61" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="62" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A62" s="13" t="inlineStr">
@@ -3091,6 +3360,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q62" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="63" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A63" s="13" t="inlineStr">
@@ -3133,6 +3407,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q63" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="64" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A64" s="13" t="inlineStr">
@@ -3175,6 +3454,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q64" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="65" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A65" s="13" t="inlineStr">
@@ -3217,6 +3501,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q65" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="66" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A66" s="13" t="inlineStr">
@@ -3259,6 +3548,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q66" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="67" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A67" s="13" t="inlineStr">
@@ -3301,6 +3595,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q67" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="68" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A68" s="13" t="inlineStr">
@@ -3343,6 +3642,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q68" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="69" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A69" s="13" t="inlineStr">
@@ -3385,6 +3689,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q69" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="70" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A70" s="13" t="inlineStr">
@@ -3427,6 +3736,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q70" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="71" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A71" s="13" t="inlineStr">
@@ -3469,6 +3783,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q71" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="72" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A72" s="13" t="inlineStr">
@@ -3511,6 +3830,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q72" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="73" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A73" s="13" t="inlineStr">
@@ -3553,6 +3877,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q73" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="74" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A74" s="13" t="inlineStr">
@@ -3595,6 +3924,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q74" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="75" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A75" s="13" t="inlineStr">
@@ -3637,6 +3971,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q75" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="76" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A76" s="13" t="inlineStr">
@@ -3679,6 +4018,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q76" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="77" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A77" s="13" t="inlineStr">
@@ -3719,6 +4063,11 @@
       <c r="P77" s="13" t="inlineStr">
         <is>
           <t>50</t>
+        </is>
+      </c>
+      <c r="Q77" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
         </is>
       </c>
     </row>
@@ -3763,6 +4112,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q78" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="79" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A79" s="13" t="inlineStr">
@@ -3805,6 +4159,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="Q79" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="80" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A80" s="13" t="inlineStr">
@@ -3847,6 +4206,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="Q80" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="81" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A81" s="13" t="inlineStr">
@@ -3889,6 +4253,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="Q81" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="82" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A82" s="13" t="inlineStr">
@@ -3931,6 +4300,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="Q82" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="83" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A83" s="13" t="inlineStr">
@@ -3973,6 +4347,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q83" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="84" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A84" s="13" t="inlineStr">
@@ -4015,6 +4394,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q84" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="85" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A85" s="13" t="inlineStr">
@@ -4057,6 +4441,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q85" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="86" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A86" s="13" t="inlineStr">
@@ -4099,6 +4488,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q86" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="87" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A87" s="13" t="inlineStr">
@@ -4141,6 +4535,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q87" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="88" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A88" s="13" t="inlineStr">
@@ -4183,6 +4582,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q88" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="89" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A89" s="13" t="inlineStr">
@@ -4225,6 +4629,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q89" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="90" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A90" s="13" t="inlineStr">
@@ -4267,6 +4676,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q90" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="91" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A91" s="13" t="inlineStr">
@@ -4309,6 +4723,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q91" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="92" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A92" s="13" t="inlineStr">
@@ -4351,6 +4770,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q92" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="93" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A93" s="13" t="inlineStr">
@@ -4393,6 +4817,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q93" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="94" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A94" s="13" t="inlineStr">
@@ -4435,6 +4864,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q94" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="95" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A95" s="13" t="inlineStr">
@@ -4477,6 +4911,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q95" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="96" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A96" s="13" t="inlineStr">
@@ -4519,6 +4958,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q96" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="97" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A97" s="13" t="inlineStr">
@@ -4561,6 +5005,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q97" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="98" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A98" s="13" t="inlineStr">
@@ -4603,6 +5052,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q98" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="99" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A99" s="13" t="inlineStr">
@@ -4645,6 +5099,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q99" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="100" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A100" s="13" t="inlineStr">
@@ -4687,6 +5146,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q100" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="101" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A101" s="13" t="inlineStr">
@@ -4729,6 +5193,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="Q101" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="102" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A102" s="13" t="inlineStr">
@@ -4771,6 +5240,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="Q102" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="103" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A103" s="13" t="inlineStr">
@@ -4813,6 +5287,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="Q103" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="104" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A104" s="13" t="inlineStr">
@@ -4855,6 +5334,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q104" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="105" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A105" s="13" t="inlineStr">
@@ -4897,6 +5381,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q105" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="106" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A106" s="13" t="inlineStr">
@@ -4939,6 +5428,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="Q106" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="107" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A107" s="13" t="inlineStr">
@@ -4981,6 +5475,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="Q107" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="108" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A108" s="13" t="inlineStr">
@@ -5023,6 +5522,11 @@
           <t>42-44</t>
         </is>
       </c>
+      <c r="Q108" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="109" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A109" s="13" t="inlineStr">
@@ -5065,6 +5569,11 @@
           <t>46-48</t>
         </is>
       </c>
+      <c r="Q109" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="110" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A110" s="13" t="inlineStr">
@@ -5107,6 +5616,11 @@
           <t>50-52</t>
         </is>
       </c>
+      <c r="Q110" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="111" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A111" s="13" t="inlineStr">
@@ -5149,6 +5663,11 @@
           <t>54-56</t>
         </is>
       </c>
+      <c r="Q111" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="112" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A112" s="13" t="inlineStr">
@@ -5191,6 +5710,11 @@
           <t>58-60</t>
         </is>
       </c>
+      <c r="Q112" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="113" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A113" s="13" t="inlineStr">
@@ -5233,6 +5757,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q113" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="114" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A114" s="13" t="inlineStr">
@@ -5275,6 +5804,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q114" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="115" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A115" s="13" t="inlineStr">
@@ -5317,6 +5851,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q115" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="116" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A116" s="13" t="inlineStr">
@@ -5359,6 +5898,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q116" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="117" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A117" s="13" t="inlineStr">
@@ -5401,6 +5945,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q117" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="118" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A118" s="13" t="inlineStr">
@@ -5443,6 +5992,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q118" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="119" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A119" s="13" t="inlineStr">
@@ -5485,6 +6039,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q119" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="120" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A120" s="13" t="inlineStr">
@@ -5527,6 +6086,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q120" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="121" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A121" s="13" t="inlineStr">
@@ -5569,6 +6133,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q121" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="122" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A122" s="13" t="inlineStr">
@@ -5611,6 +6180,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q122" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="123" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A123" s="13" t="inlineStr">
@@ -5653,6 +6227,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q123" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="124" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A124" s="13" t="inlineStr">
@@ -5695,6 +6274,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q124" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="125" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A125" s="13" t="inlineStr">
@@ -5737,6 +6321,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q125" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="126" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A126" s="13" t="inlineStr">
@@ -5779,6 +6368,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q126" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="127" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A127" s="13" t="inlineStr">
@@ -5821,6 +6415,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q127" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="128" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A128" s="13" t="inlineStr">
@@ -5863,6 +6462,11 @@
           <t>42-44</t>
         </is>
       </c>
+      <c r="Q128" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="129" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A129" s="13" t="inlineStr">
@@ -5905,6 +6509,11 @@
           <t>46-48</t>
         </is>
       </c>
+      <c r="Q129" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="130" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A130" s="13" t="inlineStr">
@@ -5947,6 +6556,11 @@
           <t>50-52</t>
         </is>
       </c>
+      <c r="Q130" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="131" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A131" s="13" t="inlineStr">
@@ -5989,6 +6603,11 @@
           <t>54-56</t>
         </is>
       </c>
+      <c r="Q131" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="132" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A132" s="13" t="inlineStr">
@@ -6031,6 +6650,11 @@
           <t>58-60</t>
         </is>
       </c>
+      <c r="Q132" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="133" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A133" s="13" t="inlineStr">
@@ -6073,6 +6697,11 @@
           <t>46-48</t>
         </is>
       </c>
+      <c r="Q133" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="134" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A134" s="13" t="inlineStr">
@@ -6115,6 +6744,11 @@
           <t>50-52</t>
         </is>
       </c>
+      <c r="Q134" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="135" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A135" s="13" t="inlineStr">
@@ -6157,6 +6791,11 @@
           <t>54-56</t>
         </is>
       </c>
+      <c r="Q135" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="136" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A136" s="13" t="inlineStr">
@@ -6199,6 +6838,11 @@
           <t>58-60</t>
         </is>
       </c>
+      <c r="Q136" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="137" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A137" s="13" t="inlineStr">
@@ -6241,6 +6885,11 @@
           <t>42-44</t>
         </is>
       </c>
+      <c r="Q137" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="138" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A138" s="13" t="inlineStr">
@@ -6283,6 +6932,11 @@
           <t>46-48</t>
         </is>
       </c>
+      <c r="Q138" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="139" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A139" s="13" t="inlineStr">
@@ -6325,6 +6979,11 @@
           <t>54-56</t>
         </is>
       </c>
+      <c r="Q139" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="140" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A140" s="13" t="inlineStr">
@@ -6367,6 +7026,11 @@
           <t>58-60</t>
         </is>
       </c>
+      <c r="Q140" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="141" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A141" s="13" t="inlineStr">
@@ -6409,6 +7073,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q141" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="142" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A142" s="13" t="inlineStr">
@@ -6451,6 +7120,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q142" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="143" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A143" s="13" t="inlineStr">
@@ -6493,6 +7167,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q143" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="144" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A144" s="13" t="inlineStr">
@@ -6535,6 +7214,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q144" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="145" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A145" s="13" t="inlineStr">
@@ -6577,6 +7261,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q145" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="146" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A146" s="13" t="inlineStr">
@@ -6619,6 +7308,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q146" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="147" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A147" s="13" t="inlineStr">
@@ -6661,6 +7355,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="Q147" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="148" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A148" s="13" t="inlineStr">
@@ -6703,6 +7402,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q148" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="149" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A149" s="13" t="inlineStr">
@@ -6745,6 +7449,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q149" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="150" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A150" s="13" t="inlineStr">
@@ -6787,6 +7496,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q150" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="151" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A151" s="13" t="inlineStr">
@@ -6829,6 +7543,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q151" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="152" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A152" s="13" t="inlineStr">
@@ -6871,6 +7590,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q152" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="153" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A153" s="13" t="inlineStr">
@@ -6913,6 +7637,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q153" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="154" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A154" s="13" t="inlineStr">
@@ -6955,6 +7684,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="Q154" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="155" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A155" s="13" t="inlineStr">
@@ -6995,6 +7729,11 @@
       <c r="P155" s="13" t="inlineStr">
         <is>
           <t>44</t>
+        </is>
+      </c>
+      <c r="Q155" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
         </is>
       </c>
     </row>
@@ -7039,6 +7778,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q156" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="157" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A157" s="13" t="inlineStr">
@@ -7081,6 +7825,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q157" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="158" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A158" s="13" t="inlineStr">
@@ -7123,6 +7872,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q158" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="159" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A159" s="13" t="inlineStr">
@@ -7165,6 +7919,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q159" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="160" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A160" s="13" t="inlineStr">
@@ -7207,6 +7966,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="Q160" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="161" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A161" s="13" t="inlineStr">
@@ -7249,6 +8013,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q161" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="162" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A162" s="13" t="inlineStr">
@@ -7291,6 +8060,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q162" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="163" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A163" s="13" t="inlineStr">
@@ -7331,6 +8105,11 @@
       <c r="P163" s="13" t="inlineStr">
         <is>
           <t>46</t>
+        </is>
+      </c>
+      <c r="Q163" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
         </is>
       </c>
     </row>
@@ -7375,6 +8154,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q164" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="165" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A165" s="13" t="inlineStr">
@@ -7417,6 +8201,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q165" s="13" t="inlineStr">
+        <is>
+          <t>Пижама</t>
+        </is>
+      </c>
     </row>
     <row r="166" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A166" s="13" t="inlineStr">
@@ -7459,6 +8248,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q166" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="167" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A167" s="13" t="inlineStr">
@@ -7501,6 +8295,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q167" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="168" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A168" s="13" t="inlineStr">
@@ -7543,6 +8342,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q168" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="169" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A169" s="13" t="inlineStr">
@@ -7585,6 +8389,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q169" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="170" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A170" s="13" t="inlineStr">
@@ -7625,6 +8434,11 @@
       <c r="P170" s="13" t="inlineStr">
         <is>
           <t>46</t>
+        </is>
+      </c>
+      <c r="Q170" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
         </is>
       </c>
     </row>
@@ -7669,6 +8483,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q171" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="172" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A172" s="13" t="inlineStr">
@@ -7711,6 +8530,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q172" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="173" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A173" s="13" t="inlineStr">
@@ -7753,6 +8577,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q173" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="174" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A174" s="13" t="inlineStr">
@@ -7795,6 +8624,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q174" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="175" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A175" s="13" t="inlineStr">
@@ -7837,6 +8671,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q175" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="176" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A176" s="13" t="inlineStr">
@@ -7879,6 +8718,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q176" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="177" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A177" s="13" t="inlineStr">
@@ -7921,6 +8765,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q177" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="178" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A178" s="13" t="inlineStr">
@@ -7963,6 +8812,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q178" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="179" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A179" s="13" t="inlineStr">
@@ -8005,6 +8859,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q179" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="180" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A180" s="13" t="inlineStr">
@@ -8047,6 +8906,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q180" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="181" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A181" s="13" t="inlineStr">
@@ -8089,6 +8953,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q181" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="182" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A182" s="13" t="inlineStr">
@@ -8131,6 +9000,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q182" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="183" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A183" s="13" t="inlineStr">
@@ -8173,6 +9047,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q183" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="184" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A184" s="13" t="inlineStr">
@@ -8215,6 +9094,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q184" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="185" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A185" s="13" t="inlineStr">
@@ -8257,6 +9141,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q185" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="186" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A186" s="13" t="inlineStr">
@@ -8299,6 +9188,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q186" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="187" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A187" s="13" t="inlineStr">
@@ -8341,6 +9235,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q187" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="188" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A188" s="13" t="inlineStr">
@@ -8383,6 +9282,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q188" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="189" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A189" s="13" t="inlineStr">
@@ -8425,6 +9329,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q189" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="190" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A190" s="13" t="inlineStr">
@@ -8467,6 +9376,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="Q190" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="191" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A191" s="13" t="inlineStr">
@@ -8509,6 +9423,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q191" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="192" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A192" s="13" t="inlineStr">
@@ -8551,6 +9470,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q192" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="193" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A193" s="13" t="inlineStr">
@@ -8593,6 +9517,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q193" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="194" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A194" s="13" t="inlineStr">
@@ -8635,6 +9564,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q194" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="195" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A195" s="13" t="inlineStr">
@@ -8677,6 +9611,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q195" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="196" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A196" s="13" t="inlineStr">
@@ -8719,6 +9658,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q196" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="197" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A197" s="13" t="inlineStr">
@@ -8761,6 +9705,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q197" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="198" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A198" s="13" t="inlineStr">
@@ -8803,6 +9752,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="Q198" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="199" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A199" s="13" t="inlineStr">
@@ -8845,6 +9799,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="Q199" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="200" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A200" s="13" t="inlineStr">
@@ -8887,6 +9846,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="Q200" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="201" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A201" s="13" t="inlineStr">
@@ -8929,6 +9893,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q201" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="202" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A202" s="13" t="inlineStr">
@@ -8971,6 +9940,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q202" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="203" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A203" s="13" t="inlineStr">
@@ -9013,6 +9987,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q203" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="204" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A204" s="13" t="inlineStr">
@@ -9053,6 +10032,11 @@
       <c r="P204" s="13" t="inlineStr">
         <is>
           <t>56</t>
+        </is>
+      </c>
+      <c r="Q204" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
         </is>
       </c>
     </row>
@@ -9097,6 +10081,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="Q205" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="206" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A206" s="13" t="inlineStr">
@@ -9139,6 +10128,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q206" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="207" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A207" s="13" t="inlineStr">
@@ -9181,6 +10175,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q207" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="208" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A208" s="13" t="inlineStr">
@@ -9223,6 +10222,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q208" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="209" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A209" s="13" t="inlineStr">
@@ -9265,6 +10269,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="Q209" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="210" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A210" s="13" t="inlineStr">
@@ -9305,6 +10314,11 @@
       <c r="P210" s="13" t="inlineStr">
         <is>
           <t>56</t>
+        </is>
+      </c>
+      <c r="Q210" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
         </is>
       </c>
     </row>
@@ -9349,6 +10363,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="Q211" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="212" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A212" s="13" t="inlineStr">
@@ -9391,6 +10410,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="Q212" s="13" t="inlineStr">
+        <is>
+          <t>Платье</t>
+        </is>
+      </c>
     </row>
     <row r="213" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A213" s="13" t="inlineStr">
@@ -9433,6 +10457,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q213" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="214" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A214" s="13" t="inlineStr">
@@ -9475,6 +10504,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q214" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="215" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A215" s="13" t="inlineStr">
@@ -9517,6 +10551,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q215" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="216" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A216" s="13" t="inlineStr">
@@ -9559,6 +10598,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q216" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="217" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A217" s="13" t="inlineStr">
@@ -9601,6 +10645,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q217" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="218" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A218" s="13" t="inlineStr">
@@ -9643,6 +10692,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="Q218" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="219" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A219" s="13" t="inlineStr">
@@ -9685,6 +10739,11 @@
           <t>110</t>
         </is>
       </c>
+      <c r="Q219" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="220" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A220" s="13" t="inlineStr">
@@ -9727,6 +10786,11 @@
           <t>116</t>
         </is>
       </c>
+      <c r="Q220" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="221" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A221" s="13" t="inlineStr">
@@ -9769,6 +10833,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="Q221" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="222" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A222" s="13" t="inlineStr">
@@ -9811,6 +10880,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="Q222" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="223" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A223" s="13" t="inlineStr">
@@ -9853,6 +10927,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="Q223" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="224" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A224" s="13" t="inlineStr">
@@ -9895,6 +10974,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="Q224" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="225" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A225" s="13" t="inlineStr">
@@ -9937,6 +11021,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="Q225" s="13" t="inlineStr">
+        <is>
+          <t>Костюм</t>
+        </is>
+      </c>
     </row>
     <row r="226" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A226" s="13" t="inlineStr">
@@ -9979,6 +11068,11 @@
           <t>42-44</t>
         </is>
       </c>
+      <c r="Q226" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="227" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A227" s="13" t="inlineStr">
@@ -10021,6 +11115,11 @@
           <t>46-48</t>
         </is>
       </c>
+      <c r="Q227" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="228" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A228" s="13" t="inlineStr">
@@ -10063,6 +11162,11 @@
           <t>50-52</t>
         </is>
       </c>
+      <c r="Q228" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="229" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A229" s="13" t="inlineStr">
@@ -10105,6 +11209,11 @@
           <t>54-56</t>
         </is>
       </c>
+      <c r="Q229" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="230" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A230" s="13" t="inlineStr">
@@ -10147,6 +11256,11 @@
           <t>42-44</t>
         </is>
       </c>
+      <c r="Q230" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="231" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A231" s="13" t="inlineStr">
@@ -10189,6 +11303,11 @@
           <t>46-48</t>
         </is>
       </c>
+      <c r="Q231" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="232" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A232" s="13" t="inlineStr">
@@ -10231,6 +11350,11 @@
           <t>50-52</t>
         </is>
       </c>
+      <c r="Q232" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="233" outlineLevel="1" ht="11" customFormat="1" customHeight="1" s="1">
       <c r="A233" s="13" t="inlineStr">
@@ -10273,6 +11397,11 @@
           <t>54-56</t>
         </is>
       </c>
+      <c r="Q233" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="234" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A234" s="13" t="inlineStr">
@@ -10315,6 +11444,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="Q234" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="235" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A235" s="13" t="inlineStr">
@@ -10357,6 +11491,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="Q235" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="236" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A236" s="13" t="inlineStr">
@@ -10399,6 +11538,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="Q236" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="237" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A237" s="13" t="inlineStr">
@@ -10441,6 +11585,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="Q237" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="238" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A238" s="13" t="inlineStr">
@@ -10483,6 +11632,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="Q238" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
+        </is>
+      </c>
     </row>
     <row r="239" outlineLevel="1" ht="12" customFormat="1" customHeight="1" s="1">
       <c r="A239" s="13" t="inlineStr">
@@ -10523,6 +11677,11 @@
       <c r="P239" s="13" t="inlineStr">
         <is>
           <t>52</t>
+        </is>
+      </c>
+      <c r="Q239" s="13" t="inlineStr">
+        <is>
+          <t>Брюки</t>
         </is>
       </c>
     </row>
@@ -10555,9 +11714,10 @@
         <v>1154</v>
       </c>
       <c r="P240" s="21" t="n"/>
+      <c r="Q240" s="21" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="469">
+  <mergeCells count="470">
     <mergeCell ref="D195:F195"/>
     <mergeCell ref="A128:C128"/>
     <mergeCell ref="D189:F189"/>
@@ -10914,6 +12074,7 @@
     <mergeCell ref="A65:C65"/>
     <mergeCell ref="D76:F76"/>
     <mergeCell ref="A80:C80"/>
+    <mergeCell ref="Q6:Q8"/>
     <mergeCell ref="A179:C179"/>
     <mergeCell ref="D28:F28"/>
     <mergeCell ref="D221:F221"/>

</xml_diff>